<commit_message>
chore: update daily scraped data
</commit_message>
<xml_diff>
--- a/arvedi_data.xlsx
+++ b/arvedi_data.xlsx
@@ -3997,7 +3997,7 @@
     </row>
     <row r="125">
       <c r="A125" t="str">
-        <v>D0144832</v>
+        <v>D0144830</v>
       </c>
       <c r="B125" t="str">
         <v>1.450</v>
@@ -4026,7 +4026,7 @@
     </row>
     <row r="126">
       <c r="A126" t="str">
-        <v>D0144830</v>
+        <v>D0144832</v>
       </c>
       <c r="B126" t="str">
         <v>1.450</v>
@@ -5041,22 +5041,22 @@
     </row>
     <row r="161">
       <c r="A161" t="str">
-        <v>D0146907</v>
+        <v>D0144821</v>
       </c>
       <c r="B161" t="str">
-        <v>1.475</v>
+        <v>1.450</v>
       </c>
       <c r="C161" t="str">
         <v>304DL</v>
       </c>
       <c r="D161" t="str">
-        <v>4.00</v>
+        <v>4.07</v>
       </c>
       <c r="E161" t="str">
-        <v>2000.000</v>
+        <v>1500.000</v>
       </c>
       <c r="F161" t="str">
-        <v>4000.000</v>
+        <v>3000.000</v>
       </c>
       <c r="G161" t="str">
         <v>SHEETS</v>
@@ -5070,22 +5070,22 @@
     </row>
     <row r="162">
       <c r="A162" t="str">
-        <v>D0144821</v>
+        <v>D0146907</v>
       </c>
       <c r="B162" t="str">
-        <v>1.450</v>
+        <v>1.475</v>
       </c>
       <c r="C162" t="str">
         <v>304DL</v>
       </c>
       <c r="D162" t="str">
-        <v>4.07</v>
+        <v>4.00</v>
       </c>
       <c r="E162" t="str">
-        <v>1500.000</v>
+        <v>2000.000</v>
       </c>
       <c r="F162" t="str">
-        <v>3000.000</v>
+        <v>4000.000</v>
       </c>
       <c r="G162" t="str">
         <v>SHEETS</v>
@@ -6317,10 +6317,10 @@
     </row>
     <row r="205">
       <c r="A205" t="str">
-        <v>D0146910</v>
+        <v>D0145959</v>
       </c>
       <c r="B205" t="str">
-        <v>1.445</v>
+        <v>790</v>
       </c>
       <c r="C205" t="str">
         <v>304DL</v>
@@ -6329,10 +6329,10 @@
         <v>4.00</v>
       </c>
       <c r="E205" t="str">
-        <v>2000.000</v>
+        <v>1250.000</v>
       </c>
       <c r="F205" t="str">
-        <v>4000.000</v>
+        <v>2500.000</v>
       </c>
       <c r="G205" t="str">
         <v>SHEETS</v>
@@ -6346,10 +6346,10 @@
     </row>
     <row r="206">
       <c r="A206" t="str">
-        <v>D0145959</v>
+        <v>D0146910</v>
       </c>
       <c r="B206" t="str">
-        <v>790</v>
+        <v>1.445</v>
       </c>
       <c r="C206" t="str">
         <v>304DL</v>
@@ -6358,10 +6358,10 @@
         <v>4.00</v>
       </c>
       <c r="E206" t="str">
-        <v>1250.000</v>
+        <v>2000.000</v>
       </c>
       <c r="F206" t="str">
-        <v>2500.000</v>
+        <v>4000.000</v>
       </c>
       <c r="G206" t="str">
         <v>SHEETS</v>
@@ -11276,10 +11276,10 @@
     </row>
     <row r="376">
       <c r="A376" t="str">
-        <v>D0147250</v>
+        <v>D0144247</v>
       </c>
       <c r="B376" t="str">
-        <v>2.533</v>
+        <v>1.260</v>
       </c>
       <c r="C376" t="str">
         <v>304DL</v>
@@ -11288,27 +11288,27 @@
         <v>0.81</v>
       </c>
       <c r="E376" t="str">
-        <v>1277.000</v>
+        <v>1250.000</v>
       </c>
       <c r="F376" t="str">
-        <v>0.000</v>
+        <v>2500.000</v>
       </c>
       <c r="G376" t="str">
-        <v>COILS</v>
+        <v>BLANKS</v>
       </c>
       <c r="H376" t="str">
         <v>BA</v>
       </c>
       <c r="I376" t="str">
-        <v>2.250</v>
+        <v>2.750</v>
       </c>
     </row>
     <row r="377">
       <c r="A377" t="str">
-        <v>D0144247</v>
+        <v>D0147250</v>
       </c>
       <c r="B377" t="str">
-        <v>1.260</v>
+        <v>2.533</v>
       </c>
       <c r="C377" t="str">
         <v>304DL</v>
@@ -11317,19 +11317,19 @@
         <v>0.81</v>
       </c>
       <c r="E377" t="str">
-        <v>1250.000</v>
+        <v>1277.000</v>
       </c>
       <c r="F377" t="str">
-        <v>2500.000</v>
+        <v>0.000</v>
       </c>
       <c r="G377" t="str">
-        <v>BLANKS</v>
+        <v>COILS</v>
       </c>
       <c r="H377" t="str">
         <v>BA</v>
       </c>
       <c r="I377" t="str">
-        <v>2.750</v>
+        <v>2.250</v>
       </c>
     </row>
     <row r="378">
@@ -12291,19 +12291,19 @@
     </row>
     <row r="411">
       <c r="A411" t="str">
-        <v>D0147416</v>
+        <v>C0925423</v>
       </c>
       <c r="B411" t="str">
-        <v>3.624</v>
+        <v>285</v>
       </c>
       <c r="C411" t="str">
         <v>304DL</v>
       </c>
       <c r="D411" t="str">
-        <v>1.00</v>
+        <v>0.61</v>
       </c>
       <c r="E411" t="str">
-        <v>500.000</v>
+        <v>80.000</v>
       </c>
       <c r="F411" t="str">
         <v>0.000</v>
@@ -12315,24 +12315,24 @@
         <v>BA</v>
       </c>
       <c r="I411" t="str">
-        <v>2.350</v>
+        <v>2.550</v>
       </c>
     </row>
     <row r="412">
       <c r="A412" t="str">
-        <v>C0925423</v>
+        <v>D0147416</v>
       </c>
       <c r="B412" t="str">
-        <v>285</v>
+        <v>3.624</v>
       </c>
       <c r="C412" t="str">
         <v>304DL</v>
       </c>
       <c r="D412" t="str">
-        <v>0.61</v>
+        <v>1.00</v>
       </c>
       <c r="E412" t="str">
-        <v>80.000</v>
+        <v>500.000</v>
       </c>
       <c r="F412" t="str">
         <v>0.000</v>
@@ -12344,7 +12344,7 @@
         <v>BA</v>
       </c>
       <c r="I412" t="str">
-        <v>2.550</v>
+        <v>2.350</v>
       </c>
     </row>
     <row r="413">
@@ -15858,7 +15858,7 @@
     </row>
     <row r="534">
       <c r="A534" t="str">
-        <v>C0970429</v>
+        <v>C0970345</v>
       </c>
       <c r="B534" t="str">
         <v>550</v>
@@ -15867,7 +15867,7 @@
         <v>316L</v>
       </c>
       <c r="D534" t="str">
-        <v>0.39</v>
+        <v>0.51</v>
       </c>
       <c r="E534" t="str">
         <v>240.000</v>
@@ -15887,7 +15887,7 @@
     </row>
     <row r="535">
       <c r="A535" t="str">
-        <v>C0970345</v>
+        <v>C0970429</v>
       </c>
       <c r="B535" t="str">
         <v>550</v>
@@ -15896,7 +15896,7 @@
         <v>316L</v>
       </c>
       <c r="D535" t="str">
-        <v>0.51</v>
+        <v>0.39</v>
       </c>
       <c r="E535" t="str">
         <v>240.000</v>
@@ -19599,19 +19599,19 @@
     </row>
     <row r="663">
       <c r="A663" t="str">
-        <v>C0905834</v>
+        <v>D0145539</v>
       </c>
       <c r="B663" t="str">
-        <v>3.888</v>
+        <v>2.120</v>
       </c>
       <c r="C663" t="str">
         <v>301NR</v>
       </c>
       <c r="D663" t="str">
-        <v>2.86</v>
+        <v>0.79</v>
       </c>
       <c r="E663" t="str">
-        <v>240.000</v>
+        <v>1272.000</v>
       </c>
       <c r="F663" t="str">
         <v>0.000</v>
@@ -19623,24 +19623,24 @@
         <v>2B</v>
       </c>
       <c r="I663" t="str">
-        <v>2.550</v>
+        <v>2.250</v>
       </c>
     </row>
     <row r="664">
       <c r="A664" t="str">
-        <v>D0145539</v>
+        <v>C0905834</v>
       </c>
       <c r="B664" t="str">
-        <v>2.120</v>
+        <v>3.888</v>
       </c>
       <c r="C664" t="str">
         <v>301NR</v>
       </c>
       <c r="D664" t="str">
-        <v>0.79</v>
+        <v>2.86</v>
       </c>
       <c r="E664" t="str">
-        <v>1272.000</v>
+        <v>240.000</v>
       </c>
       <c r="F664" t="str">
         <v>0.000</v>
@@ -19652,7 +19652,7 @@
         <v>2B</v>
       </c>
       <c r="I664" t="str">
-        <v>2.250</v>
+        <v>2.550</v>
       </c>
     </row>
     <row r="665">
@@ -20295,19 +20295,19 @@
     </row>
     <row r="687">
       <c r="A687" t="str">
-        <v>D0146574</v>
+        <v>C0984567</v>
       </c>
       <c r="B687" t="str">
-        <v>3.000</v>
+        <v>655</v>
       </c>
       <c r="C687" t="str">
         <v>409LI</v>
       </c>
       <c r="D687" t="str">
-        <v>3.06</v>
+        <v>0.50</v>
       </c>
       <c r="E687" t="str">
-        <v>1520.000</v>
+        <v>200.000</v>
       </c>
       <c r="F687" t="str">
         <v>0.000</v>
@@ -20319,24 +20319,24 @@
         <v>2B</v>
       </c>
       <c r="I687" t="str">
-        <v>1.300</v>
+        <v>1.400</v>
       </c>
     </row>
     <row r="688">
       <c r="A688" t="str">
-        <v>C0984567</v>
+        <v>D0146574</v>
       </c>
       <c r="B688" t="str">
-        <v>655</v>
+        <v>3.000</v>
       </c>
       <c r="C688" t="str">
         <v>409LI</v>
       </c>
       <c r="D688" t="str">
-        <v>0.50</v>
+        <v>3.06</v>
       </c>
       <c r="E688" t="str">
-        <v>200.000</v>
+        <v>1520.000</v>
       </c>
       <c r="F688" t="str">
         <v>0.000</v>
@@ -20348,7 +20348,7 @@
         <v>2B</v>
       </c>
       <c r="I688" t="str">
-        <v>1.400</v>
+        <v>1.300</v>
       </c>
     </row>
     <row r="689">
@@ -20643,19 +20643,19 @@
     </row>
     <row r="699">
       <c r="A699" t="str">
-        <v>D0144405</v>
+        <v>C0995208</v>
       </c>
       <c r="B699" t="str">
-        <v>1.550</v>
+        <v>1.476</v>
       </c>
       <c r="C699" t="str">
         <v>409LI</v>
       </c>
       <c r="D699" t="str">
-        <v>0.98</v>
+        <v>0.71</v>
       </c>
       <c r="E699" t="str">
-        <v>100.000</v>
+        <v>250.000</v>
       </c>
       <c r="F699" t="str">
         <v>0.000</v>
@@ -20667,24 +20667,24 @@
         <v>2B</v>
       </c>
       <c r="I699" t="str">
-        <v>1.300</v>
+        <v>1.350</v>
       </c>
     </row>
     <row r="700">
       <c r="A700" t="str">
-        <v>C0995208</v>
+        <v>D0144405</v>
       </c>
       <c r="B700" t="str">
-        <v>1.476</v>
+        <v>1.550</v>
       </c>
       <c r="C700" t="str">
         <v>409LI</v>
       </c>
       <c r="D700" t="str">
-        <v>0.71</v>
+        <v>0.98</v>
       </c>
       <c r="E700" t="str">
-        <v>250.000</v>
+        <v>100.000</v>
       </c>
       <c r="F700" t="str">
         <v>0.000</v>
@@ -20696,7 +20696,7 @@
         <v>2B</v>
       </c>
       <c r="I700" t="str">
-        <v>1.350</v>
+        <v>1.300</v>
       </c>
     </row>
     <row r="701">
@@ -24674,10 +24674,10 @@
     </row>
     <row r="838">
       <c r="A838" t="str">
-        <v>C0984604</v>
+        <v>C0967875</v>
       </c>
       <c r="B838" t="str">
-        <v>1.117</v>
+        <v>1.273</v>
       </c>
       <c r="C838" t="str">
         <v>444NB</v>
@@ -24686,7 +24686,7 @@
         <v>1.50</v>
       </c>
       <c r="E838" t="str">
-        <v>150.000</v>
+        <v>145.000</v>
       </c>
       <c r="F838" t="str">
         <v>0.000</v>
@@ -24703,10 +24703,10 @@
     </row>
     <row r="839">
       <c r="A839" t="str">
-        <v>C0967875</v>
+        <v>C0984604</v>
       </c>
       <c r="B839" t="str">
-        <v>1.273</v>
+        <v>1.117</v>
       </c>
       <c r="C839" t="str">
         <v>444NB</v>
@@ -24715,7 +24715,7 @@
         <v>1.50</v>
       </c>
       <c r="E839" t="str">
-        <v>145.000</v>
+        <v>150.000</v>
       </c>
       <c r="F839" t="str">
         <v>0.000</v>
@@ -26269,19 +26269,19 @@
     </row>
     <row r="893">
       <c r="A893" t="str">
-        <v>C0984684</v>
+        <v>C0995195</v>
       </c>
       <c r="B893" t="str">
-        <v>947</v>
+        <v>559</v>
       </c>
       <c r="C893" t="str">
         <v>439M</v>
       </c>
       <c r="D893" t="str">
-        <v>0.61</v>
+        <v>0.81</v>
       </c>
       <c r="E893" t="str">
-        <v>280.000</v>
+        <v>220.000</v>
       </c>
       <c r="F893" t="str">
         <v>0.000</v>
@@ -26298,19 +26298,19 @@
     </row>
     <row r="894">
       <c r="A894" t="str">
-        <v>C0995195</v>
+        <v>C0984684</v>
       </c>
       <c r="B894" t="str">
-        <v>559</v>
+        <v>947</v>
       </c>
       <c r="C894" t="str">
         <v>439M</v>
       </c>
       <c r="D894" t="str">
-        <v>0.81</v>
+        <v>0.61</v>
       </c>
       <c r="E894" t="str">
-        <v>220.000</v>
+        <v>280.000</v>
       </c>
       <c r="F894" t="str">
         <v>0.000</v>
@@ -28038,10 +28038,10 @@
     </row>
     <row r="954">
       <c r="A954" t="str">
-        <v>C0949117</v>
+        <v>C0991091</v>
       </c>
       <c r="B954" t="str">
-        <v>228</v>
+        <v>256</v>
       </c>
       <c r="C954" t="str">
         <v>439M</v>
@@ -28067,10 +28067,10 @@
     </row>
     <row r="955">
       <c r="A955" t="str">
-        <v>C0991091</v>
+        <v>C0949117</v>
       </c>
       <c r="B955" t="str">
-        <v>256</v>
+        <v>228</v>
       </c>
       <c r="C955" t="str">
         <v>439M</v>
@@ -30358,19 +30358,19 @@
     </row>
     <row r="1034">
       <c r="A1034" t="str">
-        <v>D0146354</v>
+        <v>C0991713</v>
       </c>
       <c r="B1034" t="str">
-        <v>3.358</v>
+        <v>1.070</v>
       </c>
       <c r="C1034" t="str">
         <v>441AR</v>
       </c>
       <c r="D1034" t="str">
-        <v>0.51</v>
+        <v>0.61</v>
       </c>
       <c r="E1034" t="str">
-        <v>220.000</v>
+        <v>300.000</v>
       </c>
       <c r="F1034" t="str">
         <v>0.000</v>
@@ -30382,24 +30382,24 @@
         <v>2B</v>
       </c>
       <c r="I1034" t="str">
-        <v>1.650</v>
+        <v>1.600</v>
       </c>
     </row>
     <row r="1035">
       <c r="A1035" t="str">
-        <v>C0991713</v>
+        <v>D0146354</v>
       </c>
       <c r="B1035" t="str">
-        <v>1.070</v>
+        <v>3.358</v>
       </c>
       <c r="C1035" t="str">
         <v>441AR</v>
       </c>
       <c r="D1035" t="str">
-        <v>0.61</v>
+        <v>0.51</v>
       </c>
       <c r="E1035" t="str">
-        <v>300.000</v>
+        <v>220.000</v>
       </c>
       <c r="F1035" t="str">
         <v>0.000</v>
@@ -30411,7 +30411,7 @@
         <v>2B</v>
       </c>
       <c r="I1035" t="str">
-        <v>1.600</v>
+        <v>1.650</v>
       </c>
     </row>
     <row r="1036">
@@ -30677,19 +30677,19 @@
     </row>
     <row r="1045">
       <c r="A1045" t="str">
-        <v>D0137215</v>
+        <v>C0967898</v>
       </c>
       <c r="B1045" t="str">
-        <v>830</v>
+        <v>459</v>
       </c>
       <c r="C1045" t="str">
         <v>441AR</v>
       </c>
       <c r="D1045" t="str">
-        <v>0.97</v>
+        <v>0.51</v>
       </c>
       <c r="E1045" t="str">
-        <v>150.000</v>
+        <v>160.000</v>
       </c>
       <c r="F1045" t="str">
         <v>0.000</v>
@@ -30701,24 +30701,24 @@
         <v>2B</v>
       </c>
       <c r="I1045" t="str">
-        <v>1.550</v>
+        <v>1.650</v>
       </c>
     </row>
     <row r="1046">
       <c r="A1046" t="str">
-        <v>C0967898</v>
+        <v>D0137215</v>
       </c>
       <c r="B1046" t="str">
-        <v>459</v>
+        <v>830</v>
       </c>
       <c r="C1046" t="str">
         <v>441AR</v>
       </c>
       <c r="D1046" t="str">
-        <v>0.51</v>
+        <v>0.97</v>
       </c>
       <c r="E1046" t="str">
-        <v>160.000</v>
+        <v>150.000</v>
       </c>
       <c r="F1046" t="str">
         <v>0.000</v>
@@ -30730,7 +30730,7 @@
         <v>2B</v>
       </c>
       <c r="I1046" t="str">
-        <v>1.650</v>
+        <v>1.550</v>
       </c>
     </row>
     <row r="1047">
@@ -31344,19 +31344,19 @@
     </row>
     <row r="1068">
       <c r="A1068" t="str">
-        <v>D0140543</v>
+        <v>D0142742</v>
       </c>
       <c r="B1068" t="str">
-        <v>269</v>
+        <v>433</v>
       </c>
       <c r="C1068" t="str">
         <v>441AR</v>
       </c>
       <c r="D1068" t="str">
-        <v>0.81</v>
+        <v>0.77</v>
       </c>
       <c r="E1068" t="str">
-        <v>120.000</v>
+        <v>215.000</v>
       </c>
       <c r="F1068" t="str">
         <v>0.000</v>
@@ -31373,19 +31373,19 @@
     </row>
     <row r="1069">
       <c r="A1069" t="str">
-        <v>D0142742</v>
+        <v>D0140543</v>
       </c>
       <c r="B1069" t="str">
-        <v>433</v>
+        <v>269</v>
       </c>
       <c r="C1069" t="str">
         <v>441AR</v>
       </c>
       <c r="D1069" t="str">
-        <v>0.77</v>
+        <v>0.81</v>
       </c>
       <c r="E1069" t="str">
-        <v>215.000</v>
+        <v>120.000</v>
       </c>
       <c r="F1069" t="str">
         <v>0.000</v>
@@ -32823,60 +32823,60 @@
     </row>
     <row r="1119">
       <c r="A1119" t="str">
-        <v>C0897501</v>
+        <v>D0144751</v>
       </c>
       <c r="B1119" t="str">
-        <v>323</v>
+        <v>1.790</v>
       </c>
       <c r="C1119" t="str">
         <v>441AR</v>
       </c>
       <c r="D1119" t="str">
-        <v>1.00</v>
+        <v>2.97</v>
       </c>
       <c r="E1119" t="str">
-        <v>70.000</v>
+        <v>1200.000</v>
       </c>
       <c r="F1119" t="str">
-        <v>0.000</v>
+        <v>1650.000</v>
       </c>
       <c r="G1119" t="str">
-        <v>COILS</v>
+        <v>BLANKS</v>
       </c>
       <c r="H1119" t="str">
         <v>2B</v>
       </c>
       <c r="I1119" t="str">
-        <v>1.600</v>
+        <v>1.800</v>
       </c>
     </row>
     <row r="1120">
       <c r="A1120" t="str">
-        <v>D0144751</v>
+        <v>C0897501</v>
       </c>
       <c r="B1120" t="str">
-        <v>1.790</v>
+        <v>323</v>
       </c>
       <c r="C1120" t="str">
         <v>441AR</v>
       </c>
       <c r="D1120" t="str">
-        <v>2.97</v>
+        <v>1.00</v>
       </c>
       <c r="E1120" t="str">
-        <v>1200.000</v>
+        <v>70.000</v>
       </c>
       <c r="F1120" t="str">
-        <v>1650.000</v>
+        <v>0.000</v>
       </c>
       <c r="G1120" t="str">
-        <v>BLANKS</v>
+        <v>COILS</v>
       </c>
       <c r="H1120" t="str">
         <v>2B</v>
       </c>
       <c r="I1120" t="str">
-        <v>1.800</v>
+        <v>1.600</v>
       </c>
     </row>
     <row r="1121">
@@ -33229,19 +33229,19 @@
     </row>
     <row r="1133">
       <c r="A1133" t="str">
-        <v>C0978487</v>
+        <v>D0142741</v>
       </c>
       <c r="B1133" t="str">
-        <v>615</v>
+        <v>428</v>
       </c>
       <c r="C1133" t="str">
         <v>441AR</v>
       </c>
       <c r="D1133" t="str">
-        <v>0.61</v>
+        <v>0.77</v>
       </c>
       <c r="E1133" t="str">
-        <v>170.000</v>
+        <v>215.000</v>
       </c>
       <c r="F1133" t="str">
         <v>0.000</v>
@@ -33253,24 +33253,24 @@
         <v>2B</v>
       </c>
       <c r="I1133" t="str">
-        <v>1.600</v>
+        <v>1.450</v>
       </c>
     </row>
     <row r="1134">
       <c r="A1134" t="str">
-        <v>D0142741</v>
+        <v>C0978487</v>
       </c>
       <c r="B1134" t="str">
-        <v>428</v>
+        <v>615</v>
       </c>
       <c r="C1134" t="str">
         <v>441AR</v>
       </c>
       <c r="D1134" t="str">
-        <v>0.77</v>
+        <v>0.61</v>
       </c>
       <c r="E1134" t="str">
-        <v>215.000</v>
+        <v>170.000</v>
       </c>
       <c r="F1134" t="str">
         <v>0.000</v>
@@ -33282,7 +33282,7 @@
         <v>2B</v>
       </c>
       <c r="I1134" t="str">
-        <v>1.450</v>
+        <v>1.600</v>
       </c>
     </row>
     <row r="1135">
@@ -35868,19 +35868,19 @@
     </row>
     <row r="1224">
       <c r="A1224" t="str">
-        <v>C0976091</v>
+        <v>C0976083</v>
       </c>
       <c r="B1224" t="str">
-        <v>346</v>
+        <v>800</v>
       </c>
       <c r="C1224" t="str">
         <v>441AR</v>
       </c>
       <c r="D1224" t="str">
-        <v>0.51</v>
+        <v>0.82</v>
       </c>
       <c r="E1224" t="str">
-        <v>160.000</v>
+        <v>130.000</v>
       </c>
       <c r="F1224" t="str">
         <v>0.000</v>
@@ -35892,24 +35892,24 @@
         <v>2B</v>
       </c>
       <c r="I1224" t="str">
-        <v>1.650</v>
+        <v>1.600</v>
       </c>
     </row>
     <row r="1225">
       <c r="A1225" t="str">
-        <v>C0976083</v>
+        <v>C0976091</v>
       </c>
       <c r="B1225" t="str">
-        <v>800</v>
+        <v>346</v>
       </c>
       <c r="C1225" t="str">
         <v>441AR</v>
       </c>
       <c r="D1225" t="str">
-        <v>0.82</v>
+        <v>0.51</v>
       </c>
       <c r="E1225" t="str">
-        <v>130.000</v>
+        <v>160.000</v>
       </c>
       <c r="F1225" t="str">
         <v>0.000</v>
@@ -35921,7 +35921,7 @@
         <v>2B</v>
       </c>
       <c r="I1225" t="str">
-        <v>1.600</v>
+        <v>1.650</v>
       </c>
     </row>
     <row r="1226">
@@ -38420,19 +38420,19 @@
     </row>
     <row r="1312">
       <c r="A1312" t="str">
-        <v>D0146550</v>
+        <v>C0991763</v>
       </c>
       <c r="B1312" t="str">
-        <v>4.600</v>
+        <v>445</v>
       </c>
       <c r="C1312" t="str">
         <v>441AR</v>
       </c>
       <c r="D1312" t="str">
-        <v>1.72</v>
+        <v>1.00</v>
       </c>
       <c r="E1312" t="str">
-        <v>1270.000</v>
+        <v>130.000</v>
       </c>
       <c r="F1312" t="str">
         <v>0.000</v>
@@ -38444,24 +38444,24 @@
         <v>2B</v>
       </c>
       <c r="I1312" t="str">
-        <v>1.700</v>
+        <v>1.600</v>
       </c>
     </row>
     <row r="1313">
       <c r="A1313" t="str">
-        <v>C0991763</v>
+        <v>D0146550</v>
       </c>
       <c r="B1313" t="str">
-        <v>445</v>
+        <v>4.600</v>
       </c>
       <c r="C1313" t="str">
         <v>441AR</v>
       </c>
       <c r="D1313" t="str">
-        <v>1.00</v>
+        <v>1.72</v>
       </c>
       <c r="E1313" t="str">
-        <v>130.000</v>
+        <v>1270.000</v>
       </c>
       <c r="F1313" t="str">
         <v>0.000</v>
@@ -38473,7 +38473,7 @@
         <v>2B</v>
       </c>
       <c r="I1313" t="str">
-        <v>1.600</v>
+        <v>1.700</v>
       </c>
     </row>
     <row r="1314">
@@ -44191,10 +44191,10 @@
     </row>
     <row r="1511">
       <c r="A1511" t="str">
-        <v>C0992428</v>
+        <v>C0976197</v>
       </c>
       <c r="B1511" t="str">
-        <v>486</v>
+        <v>500</v>
       </c>
       <c r="C1511" t="str">
         <v>4513M</v>
@@ -44203,7 +44203,7 @@
         <v>0.81</v>
       </c>
       <c r="E1511" t="str">
-        <v>100.000</v>
+        <v>103.000</v>
       </c>
       <c r="F1511" t="str">
         <v>0.000</v>
@@ -44220,10 +44220,10 @@
     </row>
     <row r="1512">
       <c r="A1512" t="str">
-        <v>C0976197</v>
+        <v>C0992428</v>
       </c>
       <c r="B1512" t="str">
-        <v>500</v>
+        <v>486</v>
       </c>
       <c r="C1512" t="str">
         <v>4513M</v>
@@ -44232,7 +44232,7 @@
         <v>0.81</v>
       </c>
       <c r="E1512" t="str">
-        <v>103.000</v>
+        <v>100.000</v>
       </c>
       <c r="F1512" t="str">
         <v>0.000</v>
@@ -48831,16 +48831,16 @@
     </row>
     <row r="1671">
       <c r="A1671" t="str">
-        <v>D0131491</v>
+        <v>C0995467</v>
       </c>
       <c r="B1671" t="str">
-        <v>2.607</v>
+        <v>3.070</v>
       </c>
       <c r="C1671" t="str">
         <v>4828</v>
       </c>
       <c r="D1671" t="str">
-        <v>1.50</v>
+        <v>1.58</v>
       </c>
       <c r="E1671" t="str">
         <v>1272.000</v>
@@ -48855,21 +48855,21 @@
         <v>2B</v>
       </c>
       <c r="I1671" t="str">
-        <v>2.750</v>
+        <v>2.850</v>
       </c>
     </row>
     <row r="1672">
       <c r="A1672" t="str">
-        <v>C0995467</v>
+        <v>D0131491</v>
       </c>
       <c r="B1672" t="str">
-        <v>3.070</v>
+        <v>2.607</v>
       </c>
       <c r="C1672" t="str">
         <v>4828</v>
       </c>
       <c r="D1672" t="str">
-        <v>1.58</v>
+        <v>1.50</v>
       </c>
       <c r="E1672" t="str">
         <v>1272.000</v>
@@ -48884,7 +48884,7 @@
         <v>2B</v>
       </c>
       <c r="I1672" t="str">
-        <v>2.850</v>
+        <v>2.750</v>
       </c>
     </row>
     <row r="1673">
@@ -49498,19 +49498,19 @@
     </row>
     <row r="1694">
       <c r="A1694" t="str">
-        <v>C0990696</v>
+        <v>D0139116</v>
       </c>
       <c r="B1694" t="str">
-        <v>1.730</v>
+        <v>4.770</v>
       </c>
       <c r="C1694" t="str">
         <v>4828</v>
       </c>
       <c r="D1694" t="str">
-        <v>1.43</v>
+        <v>1.16</v>
       </c>
       <c r="E1694" t="str">
-        <v>108.000</v>
+        <v>1272.000</v>
       </c>
       <c r="F1694" t="str">
         <v>0.000</v>
@@ -49527,19 +49527,19 @@
     </row>
     <row r="1695">
       <c r="A1695" t="str">
-        <v>D0139116</v>
+        <v>C0990696</v>
       </c>
       <c r="B1695" t="str">
-        <v>4.770</v>
+        <v>1.730</v>
       </c>
       <c r="C1695" t="str">
         <v>4828</v>
       </c>
       <c r="D1695" t="str">
-        <v>1.16</v>
+        <v>1.43</v>
       </c>
       <c r="E1695" t="str">
-        <v>1272.000</v>
+        <v>108.000</v>
       </c>
       <c r="F1695" t="str">
         <v>0.000</v>
@@ -50426,19 +50426,19 @@
     </row>
     <row r="1726">
       <c r="A1726" t="str">
-        <v>D0145926</v>
+        <v>D0147340</v>
       </c>
       <c r="B1726" t="str">
-        <v>756</v>
+        <v>5.760</v>
       </c>
       <c r="C1726" t="str">
         <v>304DL</v>
       </c>
       <c r="D1726" t="str">
-        <v>0.97</v>
+        <v>0.98</v>
       </c>
       <c r="E1726" t="str">
-        <v>240.000</v>
+        <v>1277.000</v>
       </c>
       <c r="F1726" t="str">
         <v>0.000</v>
@@ -50450,24 +50450,24 @@
         <v>2B</v>
       </c>
       <c r="I1726" t="str">
-        <v>2.250</v>
+        <v>2.350</v>
       </c>
     </row>
     <row r="1727">
       <c r="A1727" t="str">
-        <v>D0147340</v>
+        <v>D0145926</v>
       </c>
       <c r="B1727" t="str">
-        <v>5.760</v>
+        <v>756</v>
       </c>
       <c r="C1727" t="str">
         <v>304DL</v>
       </c>
       <c r="D1727" t="str">
-        <v>0.98</v>
+        <v>0.97</v>
       </c>
       <c r="E1727" t="str">
-        <v>1277.000</v>
+        <v>240.000</v>
       </c>
       <c r="F1727" t="str">
         <v>0.000</v>
@@ -50479,7 +50479,7 @@
         <v>2B</v>
       </c>
       <c r="I1727" t="str">
-        <v>2.350</v>
+        <v>2.250</v>
       </c>
     </row>
     <row r="1728">
@@ -50629,60 +50629,60 @@
     </row>
     <row r="1733">
       <c r="A1733" t="str">
-        <v>D0147033</v>
+        <v>D0147123</v>
       </c>
       <c r="B1733" t="str">
-        <v>1.575</v>
+        <v>2.370</v>
       </c>
       <c r="C1733" t="str">
         <v>304DL</v>
       </c>
       <c r="D1733" t="str">
-        <v>4.94</v>
+        <v>1.40</v>
       </c>
       <c r="E1733" t="str">
-        <v>1500.000</v>
+        <v>1522.000</v>
       </c>
       <c r="F1733" t="str">
-        <v>3000.000</v>
+        <v>0.000</v>
       </c>
       <c r="G1733" t="str">
-        <v>BLANKS</v>
+        <v>COILS</v>
       </c>
       <c r="H1733" t="str">
         <v>2B</v>
       </c>
       <c r="I1733" t="str">
-        <v>2.750</v>
+        <v>2.250</v>
       </c>
     </row>
     <row r="1734">
       <c r="A1734" t="str">
-        <v>D0147123</v>
+        <v>D0147033</v>
       </c>
       <c r="B1734" t="str">
-        <v>2.370</v>
+        <v>1.575</v>
       </c>
       <c r="C1734" t="str">
         <v>304DL</v>
       </c>
       <c r="D1734" t="str">
-        <v>1.40</v>
+        <v>4.94</v>
       </c>
       <c r="E1734" t="str">
-        <v>1522.000</v>
+        <v>1500.000</v>
       </c>
       <c r="F1734" t="str">
-        <v>0.000</v>
+        <v>3000.000</v>
       </c>
       <c r="G1734" t="str">
-        <v>COILS</v>
+        <v>BLANKS</v>
       </c>
       <c r="H1734" t="str">
         <v>2B</v>
       </c>
       <c r="I1734" t="str">
-        <v>2.250</v>
+        <v>2.750</v>
       </c>
     </row>
     <row r="1735">
@@ -51354,22 +51354,22 @@
     </row>
     <row r="1758">
       <c r="A1758" t="str">
-        <v>D0146479</v>
+        <v>D0144568</v>
       </c>
       <c r="B1758" t="str">
-        <v>980</v>
+        <v>440</v>
       </c>
       <c r="C1758" t="str">
         <v>304DL</v>
       </c>
       <c r="D1758" t="str">
-        <v>3.97</v>
+        <v>1.50</v>
       </c>
       <c r="E1758" t="str">
-        <v>1250.000</v>
+        <v>1310.000</v>
       </c>
       <c r="F1758" t="str">
-        <v>2500.000</v>
+        <v>1900.000</v>
       </c>
       <c r="G1758" t="str">
         <v>BLANKS</v>
@@ -51378,27 +51378,27 @@
         <v>2B</v>
       </c>
       <c r="I1758" t="str">
-        <v>2.750</v>
+        <v>2.350</v>
       </c>
     </row>
     <row r="1759">
       <c r="A1759" t="str">
-        <v>D0144568</v>
+        <v>D0146479</v>
       </c>
       <c r="B1759" t="str">
-        <v>440</v>
+        <v>980</v>
       </c>
       <c r="C1759" t="str">
         <v>304DL</v>
       </c>
       <c r="D1759" t="str">
-        <v>1.50</v>
+        <v>3.97</v>
       </c>
       <c r="E1759" t="str">
-        <v>1310.000</v>
+        <v>1250.000</v>
       </c>
       <c r="F1759" t="str">
-        <v>1900.000</v>
+        <v>2500.000</v>
       </c>
       <c r="G1759" t="str">
         <v>BLANKS</v>
@@ -51407,7 +51407,7 @@
         <v>2B</v>
       </c>
       <c r="I1759" t="str">
-        <v>2.350</v>
+        <v>2.750</v>
       </c>
     </row>
     <row r="1760">
@@ -52369,60 +52369,60 @@
     </row>
     <row r="1793">
       <c r="A1793" t="str">
-        <v>D0146058</v>
+        <v>D0146310</v>
       </c>
       <c r="B1793" t="str">
-        <v>2.080</v>
+        <v>1.680</v>
       </c>
       <c r="C1793" t="str">
         <v>304DL</v>
       </c>
       <c r="D1793" t="str">
-        <v>1.00</v>
+        <v>2.97</v>
       </c>
       <c r="E1793" t="str">
-        <v>1522.000</v>
+        <v>1500.000</v>
       </c>
       <c r="F1793" t="str">
-        <v>0.000</v>
+        <v>3000.000</v>
       </c>
       <c r="G1793" t="str">
-        <v>COILS</v>
+        <v>BLANKS</v>
       </c>
       <c r="H1793" t="str">
         <v>2B</v>
       </c>
       <c r="I1793" t="str">
-        <v>2.250</v>
+        <v>2.750</v>
       </c>
     </row>
     <row r="1794">
       <c r="A1794" t="str">
-        <v>D0146310</v>
+        <v>D0146058</v>
       </c>
       <c r="B1794" t="str">
-        <v>1.680</v>
+        <v>2.080</v>
       </c>
       <c r="C1794" t="str">
         <v>304DL</v>
       </c>
       <c r="D1794" t="str">
-        <v>2.97</v>
+        <v>1.00</v>
       </c>
       <c r="E1794" t="str">
-        <v>1500.000</v>
+        <v>1522.000</v>
       </c>
       <c r="F1794" t="str">
-        <v>3000.000</v>
+        <v>0.000</v>
       </c>
       <c r="G1794" t="str">
-        <v>BLANKS</v>
+        <v>COILS</v>
       </c>
       <c r="H1794" t="str">
         <v>2B</v>
       </c>
       <c r="I1794" t="str">
-        <v>2.750</v>
+        <v>2.250</v>
       </c>
     </row>
     <row r="1795">
@@ -53239,22 +53239,22 @@
     </row>
     <row r="1823">
       <c r="A1823" t="str">
-        <v>D0142622</v>
+        <v>D0146483</v>
       </c>
       <c r="B1823" t="str">
-        <v>1.520</v>
+        <v>1.470</v>
       </c>
       <c r="C1823" t="str">
         <v>304DL</v>
       </c>
       <c r="D1823" t="str">
-        <v>0.81</v>
+        <v>3.96</v>
       </c>
       <c r="E1823" t="str">
         <v>1250.000</v>
       </c>
       <c r="F1823" t="str">
-        <v>2100.000</v>
+        <v>2500.000</v>
       </c>
       <c r="G1823" t="str">
         <v>BLANKS</v>
@@ -53263,27 +53263,27 @@
         <v>2B</v>
       </c>
       <c r="I1823" t="str">
-        <v>2.450</v>
+        <v>2.750</v>
       </c>
     </row>
     <row r="1824">
       <c r="A1824" t="str">
-        <v>D0146483</v>
+        <v>D0142622</v>
       </c>
       <c r="B1824" t="str">
-        <v>1.470</v>
+        <v>1.520</v>
       </c>
       <c r="C1824" t="str">
         <v>304DL</v>
       </c>
       <c r="D1824" t="str">
-        <v>3.96</v>
+        <v>0.81</v>
       </c>
       <c r="E1824" t="str">
         <v>1250.000</v>
       </c>
       <c r="F1824" t="str">
-        <v>2500.000</v>
+        <v>2100.000</v>
       </c>
       <c r="G1824" t="str">
         <v>BLANKS</v>
@@ -53292,7 +53292,7 @@
         <v>2B</v>
       </c>
       <c r="I1824" t="str">
-        <v>2.750</v>
+        <v>2.450</v>
       </c>
     </row>
     <row r="1825">
@@ -53442,22 +53442,22 @@
     </row>
     <row r="1830">
       <c r="A1830" t="str">
-        <v>D0147180</v>
+        <v>C0991166</v>
       </c>
       <c r="B1830" t="str">
-        <v>1.552</v>
+        <v>1.300</v>
       </c>
       <c r="C1830" t="str">
         <v>304DL</v>
       </c>
       <c r="D1830" t="str">
-        <v>1.00</v>
+        <v>1.20</v>
       </c>
       <c r="E1830" t="str">
-        <v>1000.000</v>
+        <v>1250.000</v>
       </c>
       <c r="F1830" t="str">
-        <v>2000.000</v>
+        <v>2500.000</v>
       </c>
       <c r="G1830" t="str">
         <v>BLANKS</v>
@@ -53471,22 +53471,22 @@
     </row>
     <row r="1831">
       <c r="A1831" t="str">
-        <v>C0991166</v>
+        <v>D0147180</v>
       </c>
       <c r="B1831" t="str">
-        <v>1.300</v>
+        <v>1.552</v>
       </c>
       <c r="C1831" t="str">
         <v>304DL</v>
       </c>
       <c r="D1831" t="str">
-        <v>1.20</v>
+        <v>1.00</v>
       </c>
       <c r="E1831" t="str">
-        <v>1250.000</v>
+        <v>1000.000</v>
       </c>
       <c r="F1831" t="str">
-        <v>2500.000</v>
+        <v>2000.000</v>
       </c>
       <c r="G1831" t="str">
         <v>BLANKS</v>
@@ -54254,16 +54254,16 @@
     </row>
     <row r="1858">
       <c r="A1858" t="str">
-        <v>D0147418</v>
+        <v>D0147114</v>
       </c>
       <c r="B1858" t="str">
-        <v>1.070</v>
+        <v>1.999</v>
       </c>
       <c r="C1858" t="str">
         <v>304DL</v>
       </c>
       <c r="D1858" t="str">
-        <v>1.00</v>
+        <v>2.96</v>
       </c>
       <c r="E1858" t="str">
         <v>1500.000</v>
@@ -54278,21 +54278,21 @@
         <v>2B</v>
       </c>
       <c r="I1858" t="str">
-        <v>2.650</v>
+        <v>2.750</v>
       </c>
     </row>
     <row r="1859">
       <c r="A1859" t="str">
-        <v>D0147114</v>
+        <v>D0147418</v>
       </c>
       <c r="B1859" t="str">
-        <v>1.999</v>
+        <v>1.070</v>
       </c>
       <c r="C1859" t="str">
         <v>304DL</v>
       </c>
       <c r="D1859" t="str">
-        <v>2.96</v>
+        <v>1.00</v>
       </c>
       <c r="E1859" t="str">
         <v>1500.000</v>
@@ -54307,7 +54307,7 @@
         <v>2B</v>
       </c>
       <c r="I1859" t="str">
-        <v>2.750</v>
+        <v>2.650</v>
       </c>
     </row>
     <row r="1860">
@@ -56226,60 +56226,60 @@
     </row>
     <row r="1926">
       <c r="A1926" t="str">
-        <v>D0143320</v>
+        <v>D0146660</v>
       </c>
       <c r="B1926" t="str">
-        <v>530</v>
+        <v>1.150</v>
       </c>
       <c r="C1926" t="str">
         <v>304DL</v>
       </c>
       <c r="D1926" t="str">
-        <v>0.97</v>
+        <v>1.00</v>
       </c>
       <c r="E1926" t="str">
-        <v>1500.000</v>
+        <v>1277.000</v>
       </c>
       <c r="F1926" t="str">
-        <v>3000.000</v>
+        <v>0.000</v>
       </c>
       <c r="G1926" t="str">
-        <v>BLANKS</v>
+        <v>COILS</v>
       </c>
       <c r="H1926" t="str">
         <v>2B</v>
       </c>
       <c r="I1926" t="str">
-        <v>2.650</v>
+        <v>2.250</v>
       </c>
     </row>
     <row r="1927">
       <c r="A1927" t="str">
-        <v>D0146660</v>
+        <v>D0143320</v>
       </c>
       <c r="B1927" t="str">
-        <v>1.150</v>
+        <v>530</v>
       </c>
       <c r="C1927" t="str">
         <v>304DL</v>
       </c>
       <c r="D1927" t="str">
-        <v>1.00</v>
+        <v>0.97</v>
       </c>
       <c r="E1927" t="str">
-        <v>1277.000</v>
+        <v>1500.000</v>
       </c>
       <c r="F1927" t="str">
-        <v>0.000</v>
+        <v>3000.000</v>
       </c>
       <c r="G1927" t="str">
-        <v>COILS</v>
+        <v>BLANKS</v>
       </c>
       <c r="H1927" t="str">
         <v>2B</v>
       </c>
       <c r="I1927" t="str">
-        <v>2.250</v>
+        <v>2.650</v>
       </c>
     </row>
     <row r="1928">
@@ -56487,118 +56487,118 @@
     </row>
     <row r="1935">
       <c r="A1935" t="str">
-        <v>D0147209</v>
+        <v>D0147197</v>
       </c>
       <c r="B1935" t="str">
-        <v>1.554</v>
+        <v>3.834</v>
       </c>
       <c r="C1935" t="str">
         <v>304DL</v>
       </c>
       <c r="D1935" t="str">
-        <v>0.81</v>
+        <v>0.61</v>
       </c>
       <c r="E1935" t="str">
-        <v>1500.000</v>
+        <v>450.000</v>
       </c>
       <c r="F1935" t="str">
-        <v>3000.000</v>
+        <v>0.000</v>
       </c>
       <c r="G1935" t="str">
-        <v>BLANKS</v>
+        <v>COILS</v>
       </c>
       <c r="H1935" t="str">
         <v>2B</v>
       </c>
       <c r="I1935" t="str">
-        <v>2.750</v>
+        <v>2.450</v>
       </c>
     </row>
     <row r="1936">
       <c r="A1936" t="str">
-        <v>D0147197</v>
+        <v>D0147209</v>
       </c>
       <c r="B1936" t="str">
-        <v>3.834</v>
+        <v>1.554</v>
       </c>
       <c r="C1936" t="str">
         <v>304DL</v>
       </c>
       <c r="D1936" t="str">
-        <v>0.61</v>
+        <v>0.81</v>
       </c>
       <c r="E1936" t="str">
-        <v>450.000</v>
+        <v>1500.000</v>
       </c>
       <c r="F1936" t="str">
-        <v>0.000</v>
+        <v>3000.000</v>
       </c>
       <c r="G1936" t="str">
-        <v>COILS</v>
+        <v>BLANKS</v>
       </c>
       <c r="H1936" t="str">
         <v>2B</v>
       </c>
       <c r="I1936" t="str">
-        <v>2.450</v>
+        <v>2.750</v>
       </c>
     </row>
     <row r="1937">
       <c r="A1937" t="str">
-        <v>D0144189</v>
+        <v>D0147136</v>
       </c>
       <c r="B1937" t="str">
-        <v>940</v>
+        <v>490</v>
       </c>
       <c r="C1937" t="str">
         <v>304DL</v>
       </c>
       <c r="D1937" t="str">
-        <v>3.97</v>
+        <v>1.00</v>
       </c>
       <c r="E1937" t="str">
-        <v>1500.000</v>
+        <v>1000.000</v>
       </c>
       <c r="F1937" t="str">
-        <v>0.000</v>
+        <v>2000.000</v>
       </c>
       <c r="G1937" t="str">
-        <v>COILS</v>
+        <v>BLANKS</v>
       </c>
       <c r="H1937" t="str">
         <v>2B</v>
       </c>
       <c r="I1937" t="str">
-        <v>2.250</v>
+        <v>2.650</v>
       </c>
     </row>
     <row r="1938">
       <c r="A1938" t="str">
-        <v>D0147136</v>
+        <v>D0144189</v>
       </c>
       <c r="B1938" t="str">
-        <v>490</v>
+        <v>940</v>
       </c>
       <c r="C1938" t="str">
         <v>304DL</v>
       </c>
       <c r="D1938" t="str">
-        <v>1.00</v>
+        <v>3.97</v>
       </c>
       <c r="E1938" t="str">
-        <v>1000.000</v>
+        <v>1500.000</v>
       </c>
       <c r="F1938" t="str">
-        <v>2000.000</v>
+        <v>0.000</v>
       </c>
       <c r="G1938" t="str">
-        <v>BLANKS</v>
+        <v>COILS</v>
       </c>
       <c r="H1938" t="str">
         <v>2B</v>
       </c>
       <c r="I1938" t="str">
-        <v>2.650</v>
+        <v>2.250</v>
       </c>
     </row>
     <row r="1939">
@@ -56806,19 +56806,19 @@
     </row>
     <row r="1946">
       <c r="A1946" t="str">
-        <v>D0147148</v>
+        <v>D0143261</v>
       </c>
       <c r="B1946" t="str">
-        <v>1.227</v>
+        <v>790</v>
       </c>
       <c r="C1946" t="str">
         <v>304DL</v>
       </c>
       <c r="D1946" t="str">
-        <v>4.97</v>
+        <v>0.78</v>
       </c>
       <c r="E1946" t="str">
-        <v>1250.000</v>
+        <v>1277.000</v>
       </c>
       <c r="F1946" t="str">
         <v>0.000</v>
@@ -56835,19 +56835,19 @@
     </row>
     <row r="1947">
       <c r="A1947" t="str">
-        <v>D0143261</v>
+        <v>D0147148</v>
       </c>
       <c r="B1947" t="str">
-        <v>790</v>
+        <v>1.227</v>
       </c>
       <c r="C1947" t="str">
         <v>304DL</v>
       </c>
       <c r="D1947" t="str">
-        <v>0.78</v>
+        <v>4.97</v>
       </c>
       <c r="E1947" t="str">
-        <v>1277.000</v>
+        <v>1250.000</v>
       </c>
       <c r="F1947" t="str">
         <v>0.000</v>
@@ -57966,10 +57966,10 @@
     </row>
     <row r="1986">
       <c r="A1986" t="str">
-        <v>D0146186</v>
+        <v>D0145912</v>
       </c>
       <c r="B1986" t="str">
-        <v>1.715</v>
+        <v>1.520</v>
       </c>
       <c r="C1986" t="str">
         <v>304DL</v>
@@ -57978,27 +57978,27 @@
         <v>3.97</v>
       </c>
       <c r="E1986" t="str">
-        <v>1277.000</v>
+        <v>1500.000</v>
       </c>
       <c r="F1986" t="str">
-        <v>2500.000</v>
+        <v>0.000</v>
       </c>
       <c r="G1986" t="str">
-        <v>BLANKS</v>
+        <v>COILS</v>
       </c>
       <c r="H1986" t="str">
         <v>2B</v>
       </c>
       <c r="I1986" t="str">
-        <v>2.450</v>
+        <v>2.250</v>
       </c>
     </row>
     <row r="1987">
       <c r="A1987" t="str">
-        <v>D0145912</v>
+        <v>D0146186</v>
       </c>
       <c r="B1987" t="str">
-        <v>1.520</v>
+        <v>1.715</v>
       </c>
       <c r="C1987" t="str">
         <v>304DL</v>
@@ -58007,19 +58007,19 @@
         <v>3.97</v>
       </c>
       <c r="E1987" t="str">
-        <v>1500.000</v>
+        <v>1277.000</v>
       </c>
       <c r="F1987" t="str">
-        <v>0.000</v>
+        <v>2500.000</v>
       </c>
       <c r="G1987" t="str">
-        <v>COILS</v>
+        <v>BLANKS</v>
       </c>
       <c r="H1987" t="str">
         <v>2B</v>
       </c>
       <c r="I1987" t="str">
-        <v>2.250</v>
+        <v>2.450</v>
       </c>
     </row>
     <row r="1988">
@@ -58053,22 +58053,22 @@
     </row>
     <row r="1989">
       <c r="A1989" t="str">
-        <v>D0146875</v>
+        <v>D0146055</v>
       </c>
       <c r="B1989" t="str">
-        <v>905</v>
+        <v>1.374</v>
       </c>
       <c r="C1989" t="str">
         <v>304DL</v>
       </c>
       <c r="D1989" t="str">
-        <v>1.97</v>
+        <v>0.78</v>
       </c>
       <c r="E1989" t="str">
-        <v>1000.000</v>
+        <v>1500.000</v>
       </c>
       <c r="F1989" t="str">
-        <v>2000.000</v>
+        <v>3000.000</v>
       </c>
       <c r="G1989" t="str">
         <v>BLANKS</v>
@@ -58082,22 +58082,22 @@
     </row>
     <row r="1990">
       <c r="A1990" t="str">
-        <v>D0146055</v>
+        <v>D0146875</v>
       </c>
       <c r="B1990" t="str">
-        <v>1.374</v>
+        <v>905</v>
       </c>
       <c r="C1990" t="str">
         <v>304DL</v>
       </c>
       <c r="D1990" t="str">
-        <v>0.78</v>
+        <v>1.97</v>
       </c>
       <c r="E1990" t="str">
-        <v>1500.000</v>
+        <v>1000.000</v>
       </c>
       <c r="F1990" t="str">
-        <v>3000.000</v>
+        <v>2000.000</v>
       </c>
       <c r="G1990" t="str">
         <v>BLANKS</v>
@@ -60518,16 +60518,16 @@
     </row>
     <row r="2074">
       <c r="A2074" t="str">
-        <v>D0146946</v>
+        <v>D0146564</v>
       </c>
       <c r="B2074" t="str">
-        <v>1.125</v>
+        <v>1.170</v>
       </c>
       <c r="C2074" t="str">
         <v>304DL</v>
       </c>
       <c r="D2074" t="str">
-        <v>3.95</v>
+        <v>2.05</v>
       </c>
       <c r="E2074" t="str">
         <v>1500.000</v>
@@ -60547,16 +60547,16 @@
     </row>
     <row r="2075">
       <c r="A2075" t="str">
-        <v>D0146564</v>
+        <v>D0146946</v>
       </c>
       <c r="B2075" t="str">
-        <v>1.170</v>
+        <v>1.125</v>
       </c>
       <c r="C2075" t="str">
         <v>304DL</v>
       </c>
       <c r="D2075" t="str">
-        <v>2.05</v>
+        <v>3.95</v>
       </c>
       <c r="E2075" t="str">
         <v>1500.000</v>
@@ -62374,60 +62374,60 @@
     </row>
     <row r="2138">
       <c r="A2138" t="str">
-        <v>D0142306</v>
+        <v>D0145712</v>
       </c>
       <c r="B2138" t="str">
-        <v>980</v>
+        <v>1.510</v>
       </c>
       <c r="C2138" t="str">
         <v>304DL</v>
       </c>
       <c r="D2138" t="str">
-        <v>0.81</v>
+        <v>1.52</v>
       </c>
       <c r="E2138" t="str">
-        <v>1500.000</v>
+        <v>1250.000</v>
       </c>
       <c r="F2138" t="str">
-        <v>0.000</v>
+        <v>2500.000</v>
       </c>
       <c r="G2138" t="str">
-        <v>COILS</v>
+        <v>BLANKS</v>
       </c>
       <c r="H2138" t="str">
         <v>2B</v>
       </c>
       <c r="I2138" t="str">
-        <v>2.250</v>
+        <v>2.750</v>
       </c>
     </row>
     <row r="2139">
       <c r="A2139" t="str">
-        <v>D0145712</v>
+        <v>D0142306</v>
       </c>
       <c r="B2139" t="str">
-        <v>1.510</v>
+        <v>980</v>
       </c>
       <c r="C2139" t="str">
         <v>304DL</v>
       </c>
       <c r="D2139" t="str">
-        <v>1.52</v>
+        <v>0.81</v>
       </c>
       <c r="E2139" t="str">
-        <v>1250.000</v>
+        <v>1500.000</v>
       </c>
       <c r="F2139" t="str">
-        <v>2500.000</v>
+        <v>0.000</v>
       </c>
       <c r="G2139" t="str">
-        <v>BLANKS</v>
+        <v>COILS</v>
       </c>
       <c r="H2139" t="str">
         <v>2B</v>
       </c>
       <c r="I2139" t="str">
-        <v>2.750</v>
+        <v>2.250</v>
       </c>
     </row>
     <row r="2140">
@@ -62606,60 +62606,60 @@
     </row>
     <row r="2146">
       <c r="A2146" t="str">
-        <v>D0146989</v>
+        <v>D0146180</v>
       </c>
       <c r="B2146" t="str">
-        <v>775</v>
+        <v>790</v>
       </c>
       <c r="C2146" t="str">
         <v>304DL</v>
       </c>
       <c r="D2146" t="str">
-        <v>3.96</v>
+        <v>1.97</v>
       </c>
       <c r="E2146" t="str">
-        <v>1250.000</v>
+        <v>1522.000</v>
       </c>
       <c r="F2146" t="str">
-        <v>2500.000</v>
+        <v>0.000</v>
       </c>
       <c r="G2146" t="str">
-        <v>BLANKS</v>
+        <v>COILS</v>
       </c>
       <c r="H2146" t="str">
         <v>2B</v>
       </c>
       <c r="I2146" t="str">
-        <v>2.750</v>
+        <v>2.250</v>
       </c>
     </row>
     <row r="2147">
       <c r="A2147" t="str">
-        <v>D0146180</v>
+        <v>D0146989</v>
       </c>
       <c r="B2147" t="str">
-        <v>790</v>
+        <v>775</v>
       </c>
       <c r="C2147" t="str">
         <v>304DL</v>
       </c>
       <c r="D2147" t="str">
-        <v>1.97</v>
+        <v>3.96</v>
       </c>
       <c r="E2147" t="str">
-        <v>1522.000</v>
+        <v>1250.000</v>
       </c>
       <c r="F2147" t="str">
-        <v>0.000</v>
+        <v>2500.000</v>
       </c>
       <c r="G2147" t="str">
-        <v>COILS</v>
+        <v>BLANKS</v>
       </c>
       <c r="H2147" t="str">
         <v>2B</v>
       </c>
       <c r="I2147" t="str">
-        <v>2.250</v>
+        <v>2.750</v>
       </c>
     </row>
     <row r="2148">
@@ -64143,60 +64143,60 @@
     </row>
     <row r="2199">
       <c r="A2199" t="str">
-        <v>D0145857</v>
+        <v>D0147302</v>
       </c>
       <c r="B2199" t="str">
-        <v>1.416</v>
+        <v>880</v>
       </c>
       <c r="C2199" t="str">
         <v>304DL</v>
       </c>
       <c r="D2199" t="str">
-        <v>3.97</v>
+        <v>1.97</v>
       </c>
       <c r="E2199" t="str">
-        <v>1500.000</v>
+        <v>1250.000</v>
       </c>
       <c r="F2199" t="str">
-        <v>0.000</v>
+        <v>2500.000</v>
       </c>
       <c r="G2199" t="str">
-        <v>COILS</v>
+        <v>BLANKS</v>
       </c>
       <c r="H2199" t="str">
         <v>2B</v>
       </c>
       <c r="I2199" t="str">
-        <v>2.250</v>
+        <v>2.750</v>
       </c>
     </row>
     <row r="2200">
       <c r="A2200" t="str">
-        <v>D0147302</v>
+        <v>D0145857</v>
       </c>
       <c r="B2200" t="str">
-        <v>880</v>
+        <v>1.416</v>
       </c>
       <c r="C2200" t="str">
         <v>304DL</v>
       </c>
       <c r="D2200" t="str">
-        <v>1.97</v>
+        <v>3.97</v>
       </c>
       <c r="E2200" t="str">
-        <v>1250.000</v>
+        <v>1500.000</v>
       </c>
       <c r="F2200" t="str">
-        <v>2500.000</v>
+        <v>0.000</v>
       </c>
       <c r="G2200" t="str">
-        <v>BLANKS</v>
+        <v>COILS</v>
       </c>
       <c r="H2200" t="str">
         <v>2B</v>
       </c>
       <c r="I2200" t="str">
-        <v>2.750</v>
+        <v>2.250</v>
       </c>
     </row>
     <row r="2201">
@@ -64433,22 +64433,22 @@
     </row>
     <row r="2209">
       <c r="A2209" t="str">
-        <v>D0145834</v>
+        <v>D0145084</v>
       </c>
       <c r="B2209" t="str">
-        <v>1.068</v>
+        <v>360</v>
       </c>
       <c r="C2209" t="str">
         <v>304DL</v>
       </c>
       <c r="D2209" t="str">
-        <v>1.98</v>
+        <v>1.02</v>
       </c>
       <c r="E2209" t="str">
-        <v>1250.000</v>
+        <v>1500.000</v>
       </c>
       <c r="F2209" t="str">
-        <v>2500.000</v>
+        <v>3000.000</v>
       </c>
       <c r="G2209" t="str">
         <v>BLANKS</v>
@@ -64462,22 +64462,22 @@
     </row>
     <row r="2210">
       <c r="A2210" t="str">
-        <v>D0145084</v>
+        <v>D0145834</v>
       </c>
       <c r="B2210" t="str">
-        <v>360</v>
+        <v>1.068</v>
       </c>
       <c r="C2210" t="str">
         <v>304DL</v>
       </c>
       <c r="D2210" t="str">
-        <v>1.02</v>
+        <v>1.98</v>
       </c>
       <c r="E2210" t="str">
-        <v>1500.000</v>
+        <v>1250.000</v>
       </c>
       <c r="F2210" t="str">
-        <v>3000.000</v>
+        <v>2500.000</v>
       </c>
       <c r="G2210" t="str">
         <v>BLANKS</v>
@@ -65100,22 +65100,22 @@
     </row>
     <row r="2232">
       <c r="A2232" t="str">
-        <v>D0146746</v>
+        <v>D0147426</v>
       </c>
       <c r="B2232" t="str">
-        <v>535</v>
+        <v>1.565</v>
       </c>
       <c r="C2232" t="str">
         <v>304DL</v>
       </c>
       <c r="D2232" t="str">
-        <v>1.97</v>
+        <v>4.94</v>
       </c>
       <c r="E2232" t="str">
-        <v>1250.000</v>
+        <v>1500.000</v>
       </c>
       <c r="F2232" t="str">
-        <v>2500.000</v>
+        <v>3000.000</v>
       </c>
       <c r="G2232" t="str">
         <v>BLANKS</v>
@@ -65124,27 +65124,27 @@
         <v>2B</v>
       </c>
       <c r="I2232" t="str">
-        <v>2.650</v>
+        <v>2.750</v>
       </c>
     </row>
     <row r="2233">
       <c r="A2233" t="str">
-        <v>D0147426</v>
+        <v>D0146746</v>
       </c>
       <c r="B2233" t="str">
-        <v>1.565</v>
+        <v>535</v>
       </c>
       <c r="C2233" t="str">
         <v>304DL</v>
       </c>
       <c r="D2233" t="str">
-        <v>4.94</v>
+        <v>1.97</v>
       </c>
       <c r="E2233" t="str">
-        <v>1500.000</v>
+        <v>1250.000</v>
       </c>
       <c r="F2233" t="str">
-        <v>3000.000</v>
+        <v>2500.000</v>
       </c>
       <c r="G2233" t="str">
         <v>BLANKS</v>
@@ -65153,7 +65153,7 @@
         <v>2B</v>
       </c>
       <c r="I2233" t="str">
-        <v>2.750</v>
+        <v>2.650</v>
       </c>
     </row>
     <row r="2234">
@@ -65332,16 +65332,16 @@
     </row>
     <row r="2240">
       <c r="A2240" t="str">
-        <v>D0147253</v>
+        <v>D0147200</v>
       </c>
       <c r="B2240" t="str">
-        <v>718</v>
+        <v>1.560</v>
       </c>
       <c r="C2240" t="str">
         <v>304DL</v>
       </c>
       <c r="D2240" t="str">
-        <v>2.96</v>
+        <v>0.81</v>
       </c>
       <c r="E2240" t="str">
         <v>1500.000</v>
@@ -65356,21 +65356,21 @@
         <v>2B</v>
       </c>
       <c r="I2240" t="str">
-        <v>2.650</v>
+        <v>2.750</v>
       </c>
     </row>
     <row r="2241">
       <c r="A2241" t="str">
-        <v>D0147200</v>
+        <v>D0147253</v>
       </c>
       <c r="B2241" t="str">
-        <v>1.560</v>
+        <v>718</v>
       </c>
       <c r="C2241" t="str">
         <v>304DL</v>
       </c>
       <c r="D2241" t="str">
-        <v>0.81</v>
+        <v>2.96</v>
       </c>
       <c r="E2241" t="str">
         <v>1500.000</v>
@@ -65385,65 +65385,65 @@
         <v>2B</v>
       </c>
       <c r="I2241" t="str">
-        <v>2.750</v>
+        <v>2.650</v>
       </c>
     </row>
     <row r="2242">
       <c r="A2242" t="str">
-        <v>D0146306</v>
+        <v>D0143789</v>
       </c>
       <c r="B2242" t="str">
-        <v>1.680</v>
+        <v>1.830</v>
       </c>
       <c r="C2242" t="str">
         <v>304DL</v>
       </c>
       <c r="D2242" t="str">
-        <v>2.97</v>
+        <v>4.94</v>
       </c>
       <c r="E2242" t="str">
-        <v>1500.000</v>
+        <v>1522.000</v>
       </c>
       <c r="F2242" t="str">
-        <v>3000.000</v>
+        <v>0.000</v>
       </c>
       <c r="G2242" t="str">
-        <v>BLANKS</v>
+        <v>COILS</v>
       </c>
       <c r="H2242" t="str">
         <v>2B</v>
       </c>
       <c r="I2242" t="str">
-        <v>2.750</v>
+        <v>2.250</v>
       </c>
     </row>
     <row r="2243">
       <c r="A2243" t="str">
-        <v>D0143789</v>
+        <v>D0146306</v>
       </c>
       <c r="B2243" t="str">
-        <v>1.830</v>
+        <v>1.680</v>
       </c>
       <c r="C2243" t="str">
         <v>304DL</v>
       </c>
       <c r="D2243" t="str">
-        <v>4.94</v>
+        <v>2.97</v>
       </c>
       <c r="E2243" t="str">
-        <v>1522.000</v>
+        <v>1500.000</v>
       </c>
       <c r="F2243" t="str">
-        <v>0.000</v>
+        <v>3000.000</v>
       </c>
       <c r="G2243" t="str">
-        <v>COILS</v>
+        <v>BLANKS</v>
       </c>
       <c r="H2243" t="str">
         <v>2B</v>
       </c>
       <c r="I2243" t="str">
-        <v>2.250</v>
+        <v>2.750</v>
       </c>
     </row>
     <row r="2244">
@@ -65738,22 +65738,22 @@
     </row>
     <row r="2254">
       <c r="A2254" t="str">
-        <v>D0146052</v>
+        <v>D0142308</v>
       </c>
       <c r="B2254" t="str">
-        <v>1.689</v>
+        <v>1.184</v>
       </c>
       <c r="C2254" t="str">
         <v>304DL</v>
       </c>
       <c r="D2254" t="str">
-        <v>1.98</v>
+        <v>0.78</v>
       </c>
       <c r="E2254" t="str">
         <v>1000.000</v>
       </c>
       <c r="F2254" t="str">
-        <v>2000.000</v>
+        <v>2496.000</v>
       </c>
       <c r="G2254" t="str">
         <v>BLANKS</v>
@@ -65762,27 +65762,27 @@
         <v>2B</v>
       </c>
       <c r="I2254" t="str">
-        <v>2.750</v>
+        <v>2.450</v>
       </c>
     </row>
     <row r="2255">
       <c r="A2255" t="str">
-        <v>D0142308</v>
+        <v>D0146052</v>
       </c>
       <c r="B2255" t="str">
-        <v>1.184</v>
+        <v>1.689</v>
       </c>
       <c r="C2255" t="str">
         <v>304DL</v>
       </c>
       <c r="D2255" t="str">
-        <v>0.78</v>
+        <v>1.98</v>
       </c>
       <c r="E2255" t="str">
         <v>1000.000</v>
       </c>
       <c r="F2255" t="str">
-        <v>2496.000</v>
+        <v>2000.000</v>
       </c>
       <c r="G2255" t="str">
         <v>BLANKS</v>
@@ -65791,7 +65791,7 @@
         <v>2B</v>
       </c>
       <c r="I2255" t="str">
-        <v>2.450</v>
+        <v>2.750</v>
       </c>
     </row>
     <row r="2256">
@@ -70436,22 +70436,22 @@
     </row>
     <row r="2416">
       <c r="A2416" t="str">
-        <v>D0144699</v>
+        <v>D0147353</v>
       </c>
       <c r="B2416" t="str">
-        <v>1.940</v>
+        <v>570</v>
       </c>
       <c r="C2416" t="str">
         <v>316L</v>
       </c>
       <c r="D2416" t="str">
-        <v>4.97</v>
+        <v>3.96</v>
       </c>
       <c r="E2416" t="str">
-        <v>1500.000</v>
+        <v>1000.000</v>
       </c>
       <c r="F2416" t="str">
-        <v>3000.000</v>
+        <v>2000.000</v>
       </c>
       <c r="G2416" t="str">
         <v>BLANKS</v>
@@ -70460,27 +70460,27 @@
         <v>2B</v>
       </c>
       <c r="I2416" t="str">
-        <v>4.000</v>
+        <v>3.900</v>
       </c>
     </row>
     <row r="2417">
       <c r="A2417" t="str">
-        <v>D0147353</v>
+        <v>D0144699</v>
       </c>
       <c r="B2417" t="str">
-        <v>570</v>
+        <v>1.940</v>
       </c>
       <c r="C2417" t="str">
         <v>316L</v>
       </c>
       <c r="D2417" t="str">
-        <v>3.96</v>
+        <v>4.97</v>
       </c>
       <c r="E2417" t="str">
-        <v>1000.000</v>
+        <v>1500.000</v>
       </c>
       <c r="F2417" t="str">
-        <v>2000.000</v>
+        <v>3000.000</v>
       </c>
       <c r="G2417" t="str">
         <v>BLANKS</v>
@@ -70489,7 +70489,7 @@
         <v>2B</v>
       </c>
       <c r="I2417" t="str">
-        <v>3.900</v>
+        <v>4.000</v>
       </c>
     </row>
     <row r="2418">
@@ -71306,22 +71306,22 @@
     </row>
     <row r="2446">
       <c r="A2446" t="str">
-        <v>C0990727</v>
+        <v>D0146292</v>
       </c>
       <c r="B2446" t="str">
-        <v>1.500</v>
+        <v>1.342</v>
       </c>
       <c r="C2446" t="str">
         <v>316L</v>
       </c>
       <c r="D2446" t="str">
-        <v>5.08</v>
+        <v>2.96</v>
       </c>
       <c r="E2446" t="str">
-        <v>1250.000</v>
+        <v>1500.000</v>
       </c>
       <c r="F2446" t="str">
-        <v>2500.000</v>
+        <v>3000.000</v>
       </c>
       <c r="G2446" t="str">
         <v>BLANKS</v>
@@ -71330,27 +71330,27 @@
         <v>2B</v>
       </c>
       <c r="I2446" t="str">
-        <v>4.050</v>
+        <v>4.000</v>
       </c>
     </row>
     <row r="2447">
       <c r="A2447" t="str">
-        <v>D0146292</v>
+        <v>C0990727</v>
       </c>
       <c r="B2447" t="str">
-        <v>1.342</v>
+        <v>1.500</v>
       </c>
       <c r="C2447" t="str">
         <v>316L</v>
       </c>
       <c r="D2447" t="str">
-        <v>2.96</v>
+        <v>5.08</v>
       </c>
       <c r="E2447" t="str">
-        <v>1500.000</v>
+        <v>1250.000</v>
       </c>
       <c r="F2447" t="str">
-        <v>3000.000</v>
+        <v>2500.000</v>
       </c>
       <c r="G2447" t="str">
         <v>BLANKS</v>
@@ -71359,7 +71359,7 @@
         <v>2B</v>
       </c>
       <c r="I2447" t="str">
-        <v>4.000</v>
+        <v>4.050</v>
       </c>
     </row>
     <row r="2448">
@@ -72669,16 +72669,16 @@
     </row>
     <row r="2493">
       <c r="A2493" t="str">
-        <v>D0145047</v>
+        <v>D0146819</v>
       </c>
       <c r="B2493" t="str">
-        <v>2.800</v>
+        <v>1.530</v>
       </c>
       <c r="C2493" t="str">
         <v>316L</v>
       </c>
       <c r="D2493" t="str">
-        <v>1.98</v>
+        <v>0.61</v>
       </c>
       <c r="E2493" t="str">
         <v>1522.000</v>
@@ -72693,21 +72693,21 @@
         <v>2B</v>
       </c>
       <c r="I2493" t="str">
-        <v>3.500</v>
+        <v>3.600</v>
       </c>
     </row>
     <row r="2494">
       <c r="A2494" t="str">
-        <v>D0146819</v>
+        <v>D0145047</v>
       </c>
       <c r="B2494" t="str">
-        <v>1.530</v>
+        <v>2.800</v>
       </c>
       <c r="C2494" t="str">
         <v>316L</v>
       </c>
       <c r="D2494" t="str">
-        <v>0.61</v>
+        <v>1.98</v>
       </c>
       <c r="E2494" t="str">
         <v>1522.000</v>
@@ -72722,7 +72722,7 @@
         <v>2B</v>
       </c>
       <c r="I2494" t="str">
-        <v>3.600</v>
+        <v>3.500</v>
       </c>
     </row>
     <row r="2495">
@@ -73597,60 +73597,60 @@
     </row>
     <row r="2525">
       <c r="A2525" t="str">
-        <v>D0146633</v>
+        <v>D0146342</v>
       </c>
       <c r="B2525" t="str">
-        <v>1.330</v>
+        <v>2.180</v>
       </c>
       <c r="C2525" t="str">
         <v>316L</v>
       </c>
       <c r="D2525" t="str">
-        <v>2.05</v>
+        <v>0.61</v>
       </c>
       <c r="E2525" t="str">
-        <v>1000.000</v>
+        <v>130.000</v>
       </c>
       <c r="F2525" t="str">
-        <v>2000.000</v>
+        <v>0.000</v>
       </c>
       <c r="G2525" t="str">
-        <v>BLANKS</v>
+        <v>COILS</v>
       </c>
       <c r="H2525" t="str">
         <v>2B</v>
       </c>
       <c r="I2525" t="str">
-        <v>4.000</v>
+        <v>3.600</v>
       </c>
     </row>
     <row r="2526">
       <c r="A2526" t="str">
-        <v>D0146342</v>
+        <v>D0146633</v>
       </c>
       <c r="B2526" t="str">
-        <v>2.180</v>
+        <v>1.330</v>
       </c>
       <c r="C2526" t="str">
         <v>316L</v>
       </c>
       <c r="D2526" t="str">
-        <v>0.61</v>
+        <v>2.05</v>
       </c>
       <c r="E2526" t="str">
-        <v>130.000</v>
+        <v>1000.000</v>
       </c>
       <c r="F2526" t="str">
-        <v>0.000</v>
+        <v>2000.000</v>
       </c>
       <c r="G2526" t="str">
-        <v>COILS</v>
+        <v>BLANKS</v>
       </c>
       <c r="H2526" t="str">
         <v>2B</v>
       </c>
       <c r="I2526" t="str">
-        <v>3.600</v>
+        <v>4.000</v>
       </c>
     </row>
     <row r="2527">
@@ -74032,19 +74032,19 @@
     </row>
     <row r="2540">
       <c r="A2540" t="str">
-        <v>C0990894</v>
+        <v>D0146903</v>
       </c>
       <c r="B2540" t="str">
-        <v>1.534</v>
+        <v>3.990</v>
       </c>
       <c r="C2540" t="str">
         <v>316LSM</v>
       </c>
       <c r="D2540" t="str">
-        <v>1.17</v>
+        <v>1.91</v>
       </c>
       <c r="E2540" t="str">
-        <v>105.000</v>
+        <v>1272.000</v>
       </c>
       <c r="F2540" t="str">
         <v>0.000</v>
@@ -74056,24 +74056,24 @@
         <v>2B</v>
       </c>
       <c r="I2540" t="str">
-        <v>3.650</v>
+        <v>3.700</v>
       </c>
     </row>
     <row r="2541">
       <c r="A2541" t="str">
-        <v>D0146903</v>
+        <v>C0990894</v>
       </c>
       <c r="B2541" t="str">
-        <v>3.990</v>
+        <v>1.534</v>
       </c>
       <c r="C2541" t="str">
         <v>316LSM</v>
       </c>
       <c r="D2541" t="str">
-        <v>1.91</v>
+        <v>1.17</v>
       </c>
       <c r="E2541" t="str">
-        <v>1272.000</v>
+        <v>105.000</v>
       </c>
       <c r="F2541" t="str">
         <v>0.000</v>
@@ -74085,7 +74085,7 @@
         <v>2B</v>
       </c>
       <c r="I2541" t="str">
-        <v>3.700</v>
+        <v>3.650</v>
       </c>
     </row>
     <row r="2542">
@@ -77483,19 +77483,19 @@
     </row>
     <row r="2659">
       <c r="A2659" t="str">
-        <v>C0949630</v>
+        <v>C0983606</v>
       </c>
       <c r="B2659" t="str">
-        <v>1.350</v>
+        <v>2.842</v>
       </c>
       <c r="C2659" t="str">
         <v>321</v>
       </c>
       <c r="D2659" t="str">
-        <v>2.18</v>
+        <v>2.58</v>
       </c>
       <c r="E2659" t="str">
-        <v>160.000</v>
+        <v>220.000</v>
       </c>
       <c r="F2659" t="str">
         <v>0.000</v>
@@ -77512,19 +77512,19 @@
     </row>
     <row r="2660">
       <c r="A2660" t="str">
-        <v>C0983606</v>
+        <v>C0949630</v>
       </c>
       <c r="B2660" t="str">
-        <v>2.842</v>
+        <v>1.350</v>
       </c>
       <c r="C2660" t="str">
         <v>321</v>
       </c>
       <c r="D2660" t="str">
-        <v>2.58</v>
+        <v>2.18</v>
       </c>
       <c r="E2660" t="str">
-        <v>220.000</v>
+        <v>160.000</v>
       </c>
       <c r="F2660" t="str">
         <v>0.000</v>
@@ -77715,19 +77715,19 @@
     </row>
     <row r="2667">
       <c r="A2667" t="str">
-        <v>C0928551</v>
+        <v>C0967732</v>
       </c>
       <c r="B2667" t="str">
-        <v>676</v>
+        <v>3.732</v>
       </c>
       <c r="C2667" t="str">
         <v>321</v>
       </c>
       <c r="D2667" t="str">
-        <v>1.51</v>
+        <v>2.58</v>
       </c>
       <c r="E2667" t="str">
-        <v>90.000</v>
+        <v>235.000</v>
       </c>
       <c r="F2667" t="str">
         <v>0.000</v>
@@ -77739,24 +77739,24 @@
         <v>2B</v>
       </c>
       <c r="I2667" t="str">
-        <v>2.450</v>
+        <v>2.650</v>
       </c>
     </row>
     <row r="2668">
       <c r="A2668" t="str">
-        <v>C0967732</v>
+        <v>C0928551</v>
       </c>
       <c r="B2668" t="str">
-        <v>3.732</v>
+        <v>676</v>
       </c>
       <c r="C2668" t="str">
         <v>321</v>
       </c>
       <c r="D2668" t="str">
-        <v>2.58</v>
+        <v>1.51</v>
       </c>
       <c r="E2668" t="str">
-        <v>235.000</v>
+        <v>90.000</v>
       </c>
       <c r="F2668" t="str">
         <v>0.000</v>
@@ -77768,7 +77768,7 @@
         <v>2B</v>
       </c>
       <c r="I2668" t="str">
-        <v>2.650</v>
+        <v>2.450</v>
       </c>
     </row>
     <row r="2669">
@@ -78817,77 +78817,77 @@
     </row>
     <row r="2705">
       <c r="A2705" t="str">
-        <v>D0146199</v>
+        <v>C0967720</v>
       </c>
       <c r="B2705" t="str">
-        <v>565</v>
+        <v>934</v>
       </c>
       <c r="C2705" t="str">
         <v>321</v>
       </c>
       <c r="D2705" t="str">
-        <v>2.08</v>
+        <v>1.19</v>
       </c>
       <c r="E2705" t="str">
-        <v>1250.000</v>
+        <v>80.000</v>
       </c>
       <c r="F2705" t="str">
-        <v>2500.000</v>
+        <v>0.000</v>
       </c>
       <c r="G2705" t="str">
-        <v>BLANKS</v>
+        <v>COILS</v>
       </c>
       <c r="H2705" t="str">
         <v>2B</v>
       </c>
       <c r="I2705" t="str">
-        <v>2.750</v>
+        <v>2.450</v>
       </c>
     </row>
     <row r="2706">
       <c r="A2706" t="str">
-        <v>C0898763</v>
+        <v>D0146199</v>
       </c>
       <c r="B2706" t="str">
-        <v>6.830</v>
+        <v>565</v>
       </c>
       <c r="C2706" t="str">
         <v>321</v>
       </c>
       <c r="D2706" t="str">
-        <v>2.58</v>
+        <v>2.08</v>
       </c>
       <c r="E2706" t="str">
-        <v>430.000</v>
+        <v>1250.000</v>
       </c>
       <c r="F2706" t="str">
-        <v>0.000</v>
+        <v>2500.000</v>
       </c>
       <c r="G2706" t="str">
-        <v>COILS</v>
+        <v>BLANKS</v>
       </c>
       <c r="H2706" t="str">
         <v>2B</v>
       </c>
       <c r="I2706" t="str">
-        <v>2.650</v>
+        <v>2.750</v>
       </c>
     </row>
     <row r="2707">
       <c r="A2707" t="str">
-        <v>C0967720</v>
+        <v>C0898763</v>
       </c>
       <c r="B2707" t="str">
-        <v>934</v>
+        <v>6.830</v>
       </c>
       <c r="C2707" t="str">
         <v>321</v>
       </c>
       <c r="D2707" t="str">
-        <v>1.19</v>
+        <v>2.58</v>
       </c>
       <c r="E2707" t="str">
-        <v>80.000</v>
+        <v>430.000</v>
       </c>
       <c r="F2707" t="str">
         <v>0.000</v>
@@ -78899,7 +78899,7 @@
         <v>2B</v>
       </c>
       <c r="I2707" t="str">
-        <v>2.450</v>
+        <v>2.650</v>
       </c>
     </row>
     <row r="2708">

</xml_diff>